<commit_message>
Add 14 completed orders from 21/10 export (rolls to be set by hand); Halishahar ones to Collegiate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Student data.xlsx
+++ b/Student data.xlsx
@@ -17,9 +17,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm"/>
-    <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -502,7 +502,7 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
@@ -511,7 +511,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
@@ -647,7 +647,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -719,7 +719,8 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1134,7 +1135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S286"/>
+  <dimension ref="A1:S300"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.5648148148148" customWidth="1" style="22" min="1" max="1"/>
@@ -21706,1136 +21707,2200 @@
       </c>
     </row>
     <row r="272">
-      <c r="A272" t="n">
+      <c r="A272" s="4" t="n">
         <v>3843</v>
       </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
+      <c r="B272" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C272" s="4" t="inlineStr">
         <is>
           <t>01720601933</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr">
+      <c r="D272" s="4" t="inlineStr">
         <is>
           <t>DJE2WL950U</t>
         </is>
       </c>
-      <c r="G272" s="27" t="n">
+      <c r="G272" s="28" t="n">
         <v>46309.30418981481</v>
       </c>
-      <c r="H272" t="inlineStr">
+      <c r="H272" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I272" t="inlineStr">
+      <c r="I272" s="4" t="inlineStr">
         <is>
           <t>Safwan Zaman Ahnaf</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr">
+      <c r="J272" s="4" t="inlineStr">
         <is>
           <t>সাফওয়ান জামান আহনাফ</t>
         </is>
       </c>
-      <c r="K272" t="inlineStr">
+      <c r="K272" s="4" t="inlineStr">
         <is>
           <t>Md Shahiduzzaman</t>
         </is>
       </c>
-      <c r="L272" t="inlineStr">
+      <c r="L272" s="4" t="inlineStr">
         <is>
           <t>Tahmina Siddeka</t>
         </is>
       </c>
-      <c r="M272" t="inlineStr">
+      <c r="M272" s="4" t="inlineStr">
         <is>
           <t>Delta School and College</t>
         </is>
       </c>
-      <c r="N272" t="n">
+      <c r="N272" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="O272" t="n">
+      <c r="O272" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P272" t="inlineStr">
+      <c r="P272" s="4" t="inlineStr">
         <is>
           <t>Bakolia Access Road, Bakolia, Chattogram</t>
         </is>
       </c>
-      <c r="Q272" t="inlineStr">
+      <c r="Q272" s="4" t="inlineStr">
         <is>
           <t>01850401816</t>
         </is>
       </c>
-      <c r="S272" t="inlineStr">
+      <c r="S272" s="4" t="inlineStr">
         <is>
           <t>dewanhat</t>
         </is>
       </c>
     </row>
     <row r="273">
-      <c r="A273" t="n">
+      <c r="A273" s="4" t="n">
         <v>3844</v>
       </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C273" t="inlineStr">
+      <c r="B273" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C273" s="4" t="inlineStr">
         <is>
           <t>01815287418</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
+      <c r="D273" s="4" t="inlineStr">
         <is>
           <t>DJE90HFF6V</t>
         </is>
       </c>
-      <c r="G273" s="27" t="n">
+      <c r="G273" s="28" t="n">
         <v>46309.67502314815</v>
       </c>
-      <c r="H273" t="inlineStr">
+      <c r="H273" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I273" t="inlineStr">
+      <c r="I273" s="4" t="inlineStr">
         <is>
           <t>Twasin Alam</t>
         </is>
       </c>
-      <c r="J273" t="inlineStr">
+      <c r="J273" s="4" t="inlineStr">
         <is>
           <t>ত্বসীন আলম</t>
         </is>
       </c>
-      <c r="K273" t="inlineStr">
+      <c r="K273" s="4" t="inlineStr">
         <is>
           <t>Md. Khurshidul Alam</t>
         </is>
       </c>
-      <c r="L273" t="inlineStr">
+      <c r="L273" s="4" t="inlineStr">
         <is>
           <t>Mst. Yesmin Akter</t>
         </is>
       </c>
-      <c r="M273" t="inlineStr">
+      <c r="M273" s="4" t="inlineStr">
         <is>
           <t>Chattogram Collegiate School</t>
         </is>
       </c>
-      <c r="N273" t="n">
+      <c r="N273" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="O273" t="n">
+      <c r="O273" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="P273" t="inlineStr">
+      <c r="P273" s="4" t="inlineStr">
         <is>
           <t>Nayabazar, Halishahar, Chattogram.</t>
         </is>
       </c>
-      <c r="Q273" t="inlineStr">
+      <c r="Q273" s="4" t="inlineStr">
         <is>
           <t>01815287418</t>
         </is>
       </c>
-      <c r="S273" t="inlineStr">
+      <c r="S273" s="4" t="inlineStr">
         <is>
           <t>halishahar</t>
         </is>
       </c>
     </row>
     <row r="274">
-      <c r="A274" t="n">
+      <c r="A274" s="4" t="n">
         <v>3846</v>
       </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr">
+      <c r="B274" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C274" s="4" t="inlineStr">
         <is>
           <t>01722966006</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr">
+      <c r="D274" s="4" t="inlineStr">
         <is>
           <t>DJF712IC31</t>
         </is>
       </c>
-      <c r="G274" s="27" t="n">
+      <c r="G274" s="28" t="n">
         <v>46310.18609953704</v>
       </c>
-      <c r="H274" t="inlineStr">
+      <c r="H274" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I274" t="inlineStr">
+      <c r="I274" s="4" t="inlineStr">
         <is>
           <t>Md.Ridowan Bin Arif</t>
         </is>
       </c>
-      <c r="J274" t="inlineStr">
+      <c r="J274" s="4" t="inlineStr">
         <is>
           <t>মোঃ রিদওয়ান বিন আরিফ</t>
         </is>
       </c>
-      <c r="K274" t="inlineStr">
+      <c r="K274" s="4" t="inlineStr">
         <is>
           <t>Md.Ariful Islam</t>
         </is>
       </c>
-      <c r="L274" t="inlineStr">
+      <c r="L274" s="4" t="inlineStr">
         <is>
           <t>Rikta Akter</t>
         </is>
       </c>
-      <c r="M274" t="inlineStr">
+      <c r="M274" s="4" t="inlineStr">
         <is>
           <t>মোঃ আরিফুল ইসলাম</t>
         </is>
       </c>
-      <c r="N274" t="inlineStr">
+      <c r="N274" s="4" t="inlineStr">
         <is>
           <t>Seven</t>
         </is>
       </c>
-      <c r="O274" t="n">
+      <c r="O274" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="P274" t="inlineStr">
+      <c r="P274" s="4" t="inlineStr">
         <is>
           <t>Sadarghat, Chittagong</t>
         </is>
       </c>
-      <c r="Q274" t="inlineStr">
+      <c r="Q274" s="4" t="inlineStr">
         <is>
           <t>01722966006</t>
         </is>
       </c>
-      <c r="S274" t="inlineStr">
+      <c r="S274" s="4" t="inlineStr">
         <is>
           <t>dewanhat</t>
         </is>
       </c>
     </row>
     <row r="275">
-      <c r="A275" t="n">
+      <c r="A275" s="4" t="n">
         <v>3847</v>
       </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C275" t="inlineStr">
+      <c r="B275" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C275" s="4" t="inlineStr">
         <is>
           <t>01319004461</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr">
+      <c r="D275" s="4" t="inlineStr">
         <is>
           <t>DJF01W6ENE</t>
         </is>
       </c>
-      <c r="G275" s="27" t="n">
+      <c r="G275" s="28" t="n">
         <v>46310.52702546296</v>
       </c>
-      <c r="H275" t="inlineStr">
+      <c r="H275" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I275" t="inlineStr">
+      <c r="I275" s="4" t="inlineStr">
         <is>
           <t>AHMAD JAHEE</t>
         </is>
       </c>
-      <c r="J275" t="inlineStr">
+      <c r="J275" s="4" t="inlineStr">
         <is>
           <t>আহমাদ জাহী</t>
         </is>
       </c>
-      <c r="K275" t="inlineStr">
+      <c r="K275" s="4" t="inlineStr">
         <is>
           <t>JALAL UDDIN</t>
         </is>
       </c>
-      <c r="L275" t="inlineStr">
+      <c r="L275" s="4" t="inlineStr">
         <is>
           <t>SHAMIM AKTER</t>
         </is>
       </c>
-      <c r="M275" t="inlineStr">
+      <c r="M275" s="4" t="inlineStr">
         <is>
           <t>CHATTOGRAM COLLEGIATE SCHOOL</t>
         </is>
       </c>
-      <c r="N275" t="inlineStr">
+      <c r="N275" s="4" t="inlineStr">
         <is>
           <t>FIVE</t>
         </is>
       </c>
-      <c r="O275" t="n">
+      <c r="O275" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="P275" t="inlineStr">
+      <c r="P275" s="4" t="inlineStr">
         <is>
           <t>30 NO. M M ALI ROAD, LALKHAN BAZAR, VOTAIYA COLONY, DAMPARA-4000, KHULSHI, CHATTOGRAM</t>
         </is>
       </c>
-      <c r="Q275" t="inlineStr">
+      <c r="Q275" s="4" t="inlineStr">
         <is>
           <t>01626914730</t>
         </is>
       </c>
-      <c r="S275" t="inlineStr">
+      <c r="S275" s="4" t="inlineStr">
         <is>
           <t>dewanhat</t>
         </is>
       </c>
     </row>
     <row r="276">
-      <c r="A276" t="n">
+      <c r="A276" s="4" t="n">
         <v>3848</v>
       </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="E276" t="inlineStr">
+      <c r="B276" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E276" s="4" t="inlineStr">
         <is>
           <t>01723088207</t>
         </is>
       </c>
-      <c r="F276" t="inlineStr">
+      <c r="F276" s="4" t="inlineStr">
         <is>
           <t>7659Q5GH</t>
         </is>
       </c>
-      <c r="G276" s="27" t="n">
+      <c r="G276" s="28" t="n">
         <v>46310.56505787037</v>
       </c>
-      <c r="H276" t="inlineStr">
+      <c r="H276" s="4" t="inlineStr">
         <is>
           <t>Girl</t>
         </is>
       </c>
-      <c r="I276" t="inlineStr">
+      <c r="I276" s="4" t="inlineStr">
         <is>
           <t>Nusrat Jahan</t>
         </is>
       </c>
-      <c r="J276" t="inlineStr">
+      <c r="J276" s="4" t="inlineStr">
         <is>
           <t>নুসরাত জাহান</t>
         </is>
       </c>
-      <c r="K276" t="inlineStr">
+      <c r="K276" s="4" t="inlineStr">
         <is>
           <t>Mohammed Jafor Iqbal Talukder</t>
         </is>
       </c>
-      <c r="L276" t="inlineStr">
+      <c r="L276" s="4" t="inlineStr">
         <is>
           <t>Saleha Akter</t>
         </is>
       </c>
-      <c r="M276" t="inlineStr">
+      <c r="M276" s="4" t="inlineStr">
         <is>
           <t>CDDL Navy School</t>
         </is>
       </c>
-      <c r="N276" t="inlineStr">
+      <c r="N276" s="4" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="O276" t="inlineStr">
+      <c r="O276" s="4" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="P276" t="inlineStr">
+      <c r="P276" s="4" t="inlineStr">
         <is>
           <t>Rubi cement colony,(Rab 7 এর পাশে),North Patenga,Chattogram</t>
         </is>
       </c>
-      <c r="Q276" t="inlineStr">
+      <c r="Q276" s="4" t="inlineStr">
         <is>
           <t>01336826867</t>
         </is>
       </c>
-      <c r="S276" t="inlineStr">
+      <c r="S276" s="4" t="inlineStr">
         <is>
           <t>Patenga</t>
         </is>
       </c>
     </row>
     <row r="277">
-      <c r="A277" t="n">
+      <c r="A277" s="4" t="n">
         <v>3849</v>
       </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C277" t="inlineStr">
+      <c r="B277" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C277" s="4" t="inlineStr">
         <is>
           <t>01723088207</t>
         </is>
       </c>
-      <c r="D277" t="inlineStr">
+      <c r="D277" s="4" t="inlineStr">
         <is>
           <t>DJF424TGIU</t>
         </is>
       </c>
-      <c r="G277" s="27" t="n">
+      <c r="G277" s="28" t="n">
         <v>46310.60385416666</v>
       </c>
-      <c r="H277" t="inlineStr">
+      <c r="H277" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I277" t="inlineStr">
+      <c r="I277" s="4" t="inlineStr">
         <is>
           <t>Md.Samiul Islam Alvi</t>
         </is>
       </c>
-      <c r="J277" t="inlineStr">
+      <c r="J277" s="4" t="inlineStr">
         <is>
           <t>মো:সামিউল ইসলাম আলভী</t>
         </is>
       </c>
-      <c r="K277" t="inlineStr">
+      <c r="K277" s="4" t="inlineStr">
         <is>
           <t>Md Saiful Islam</t>
         </is>
       </c>
-      <c r="L277" t="inlineStr">
+      <c r="L277" s="4" t="inlineStr">
         <is>
           <t>Sarmeen Akter</t>
         </is>
       </c>
-      <c r="M277" t="inlineStr">
+      <c r="M277" s="4" t="inlineStr">
         <is>
           <t>Ispahani Public School And College</t>
         </is>
       </c>
-      <c r="N277" t="inlineStr">
+      <c r="N277" s="4" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="O277" t="n">
+      <c r="O277" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="P277" t="inlineStr">
+      <c r="P277" s="4" t="inlineStr">
         <is>
           <t>Shah Garibullah Housing Society,Road no.1/1,House no.01,Khulshi. Chattogram</t>
         </is>
       </c>
-      <c r="Q277" t="inlineStr">
+      <c r="Q277" s="4" t="inlineStr">
         <is>
           <t>01717944271</t>
         </is>
       </c>
-      <c r="S277" t="inlineStr">
+      <c r="S277" s="4" t="inlineStr">
         <is>
           <t>agrabad</t>
         </is>
       </c>
     </row>
     <row r="278">
-      <c r="A278" t="n">
+      <c r="A278" s="4" t="n">
         <v>3850</v>
       </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
+      <c r="B278" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C278" s="4" t="inlineStr">
         <is>
           <t>01521735429</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr">
+      <c r="D278" s="4" t="inlineStr">
         <is>
           <t>DJG53FJD7N</t>
         </is>
       </c>
-      <c r="G278" s="27" t="n">
+      <c r="G278" s="28" t="n">
         <v>46311.44094907407</v>
       </c>
-      <c r="H278" t="inlineStr">
+      <c r="H278" s="4" t="inlineStr">
         <is>
           <t>Girl</t>
         </is>
       </c>
-      <c r="I278" t="inlineStr">
+      <c r="I278" s="4" t="inlineStr">
         <is>
           <t>Tasnia Farin Yusha</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr">
+      <c r="J278" s="4" t="inlineStr">
         <is>
           <t>তাসনিয়া ফারিন ইউশা</t>
         </is>
       </c>
-      <c r="K278" t="inlineStr">
+      <c r="K278" s="4" t="inlineStr">
         <is>
           <t>Mohammad Mojibul Hoque</t>
         </is>
       </c>
-      <c r="L278" t="inlineStr">
+      <c r="L278" s="4" t="inlineStr">
         <is>
           <t>Nilufer Yeasmin</t>
         </is>
       </c>
-      <c r="M278" t="inlineStr">
+      <c r="M278" s="4" t="inlineStr">
         <is>
           <t>Dr. Khastagir Govt. Girls High School</t>
         </is>
       </c>
-      <c r="N278" t="n">
+      <c r="N278" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O278" t="n">
+      <c r="O278" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="P278" t="inlineStr">
+      <c r="P278" s="4" t="inlineStr">
         <is>
           <t>271, Rosulbag C Block, Bakolia, Chattogram</t>
         </is>
       </c>
-      <c r="Q278" t="n">
+      <c r="Q278" s="4" t="n">
         <v>8801970433883</v>
       </c>
-      <c r="S278" t="inlineStr">
+      <c r="S278" s="4" t="inlineStr">
         <is>
           <t>dewanhat</t>
         </is>
       </c>
     </row>
     <row r="279">
-      <c r="A279" t="n">
+      <c r="A279" s="4" t="n">
         <v>3852</v>
       </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C279" t="inlineStr">
+      <c r="B279" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C279" s="4" t="inlineStr">
         <is>
           <t>01612938480</t>
         </is>
       </c>
-      <c r="D279" t="inlineStr">
+      <c r="D279" s="4" t="inlineStr">
         <is>
           <t>DJG93UQR9T</t>
         </is>
       </c>
-      <c r="G279" s="27" t="n">
+      <c r="G279" s="28" t="n">
         <v>46311.6040625</v>
       </c>
-      <c r="H279" t="inlineStr">
+      <c r="H279" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I279" t="inlineStr">
+      <c r="I279" s="4" t="inlineStr">
         <is>
           <t>Prantik Barua Dhrubo</t>
         </is>
       </c>
-      <c r="J279" t="inlineStr">
+      <c r="J279" s="4" t="inlineStr">
         <is>
           <t>প্রান্তিক বড়ুয়া ধ্রুব</t>
         </is>
       </c>
-      <c r="K279" t="inlineStr">
+      <c r="K279" s="4" t="inlineStr">
         <is>
           <t>Dipak Barua</t>
         </is>
       </c>
-      <c r="L279" t="inlineStr">
+      <c r="L279" s="4" t="inlineStr">
         <is>
           <t>Priya Barua</t>
         </is>
       </c>
-      <c r="M279" t="inlineStr">
+      <c r="M279" s="4" t="inlineStr">
         <is>
           <t>Green Bell School &amp; College</t>
         </is>
       </c>
-      <c r="N279" t="inlineStr">
+      <c r="N279" s="4" t="inlineStr">
         <is>
           <t>Class Six</t>
         </is>
       </c>
-      <c r="O279" t="inlineStr">
+      <c r="O279" s="4" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="P279" t="inlineStr">
+      <c r="P279" s="4" t="inlineStr">
         <is>
           <t>Dhum para Khatgor Pategha Chattagram</t>
         </is>
       </c>
-      <c r="Q279" t="inlineStr">
+      <c r="Q279" s="4" t="inlineStr">
         <is>
           <t>01612938480</t>
         </is>
       </c>
-      <c r="S279" t="inlineStr">
+      <c r="S279" s="4" t="inlineStr">
         <is>
           <t>Patenga</t>
         </is>
       </c>
     </row>
     <row r="280">
-      <c r="A280" t="n">
+      <c r="A280" s="4" t="n">
         <v>3853</v>
       </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C280" t="inlineStr">
+      <c r="B280" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C280" s="4" t="inlineStr">
         <is>
           <t>01300480754</t>
         </is>
       </c>
-      <c r="D280" t="inlineStr">
+      <c r="D280" s="4" t="inlineStr">
         <is>
           <t>DJG73Z172T</t>
         </is>
       </c>
-      <c r="G280" s="27" t="n">
+      <c r="G280" s="28" t="n">
         <v>46311.64581018518</v>
       </c>
-      <c r="H280" t="inlineStr">
+      <c r="H280" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I280" t="inlineStr">
+      <c r="I280" s="4" t="inlineStr">
         <is>
           <t>MD.Rayhan Alam</t>
         </is>
       </c>
-      <c r="J280" t="inlineStr">
+      <c r="J280" s="4" t="inlineStr">
         <is>
           <t>মোঃ রায়হান আলম</t>
         </is>
       </c>
-      <c r="K280" t="inlineStr">
+      <c r="K280" s="4" t="inlineStr">
         <is>
           <t>Jahangir Alam</t>
         </is>
       </c>
-      <c r="L280" t="inlineStr">
+      <c r="L280" s="4" t="inlineStr">
         <is>
           <t>Rehana Akther</t>
         </is>
       </c>
-      <c r="M280" t="inlineStr">
+      <c r="M280" s="4" t="inlineStr">
         <is>
           <t>Chattogram Collegiate School, Chattogram</t>
         </is>
       </c>
-      <c r="N280" t="n">
+      <c r="N280" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="O280" t="n">
+      <c r="O280" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="P280" t="inlineStr">
+      <c r="P280" s="4" t="inlineStr">
         <is>
           <t>AK house 121, Chandanpura, Chawk bazar, Chattogram</t>
         </is>
       </c>
-      <c r="Q280" t="inlineStr">
+      <c r="Q280" s="4" t="inlineStr">
         <is>
           <t>01851911435</t>
         </is>
       </c>
-      <c r="S280" t="inlineStr">
+      <c r="S280" s="4" t="inlineStr">
         <is>
           <t>dewanhat</t>
         </is>
       </c>
     </row>
     <row r="281">
-      <c r="A281" t="n">
+      <c r="A281" s="4" t="n">
         <v>3854</v>
       </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C281" t="inlineStr">
+      <c r="B281" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C281" s="4" t="inlineStr">
         <is>
           <t>01873029849</t>
         </is>
       </c>
-      <c r="D281" t="inlineStr">
+      <c r="D281" s="4" t="inlineStr">
         <is>
           <t>DJG541N0CZ</t>
         </is>
       </c>
-      <c r="G281" s="27" t="n">
+      <c r="G281" s="28" t="n">
         <v>46311.66945601852</v>
       </c>
-      <c r="H281" t="inlineStr">
+      <c r="H281" s="4" t="inlineStr">
         <is>
           <t>Girl</t>
         </is>
       </c>
-      <c r="I281" t="inlineStr">
+      <c r="I281" s="4" t="inlineStr">
         <is>
           <t>Fahmida khanom alifa</t>
         </is>
       </c>
-      <c r="J281" t="inlineStr">
+      <c r="J281" s="4" t="inlineStr">
         <is>
           <t>ফাহমিদা খানম আলিফা</t>
         </is>
       </c>
-      <c r="K281" t="inlineStr">
+      <c r="K281" s="4" t="inlineStr">
         <is>
           <t>Ayub khan</t>
         </is>
       </c>
-      <c r="L281" t="inlineStr">
+      <c r="L281" s="4" t="inlineStr">
         <is>
           <t>Firoja akther</t>
         </is>
       </c>
-      <c r="M281" t="inlineStr">
+      <c r="M281" s="4" t="inlineStr">
         <is>
           <t>South kattali pran hori model gov't primary school</t>
         </is>
       </c>
-      <c r="N281" t="inlineStr">
+      <c r="N281" s="4" t="inlineStr">
         <is>
           <t>Five</t>
         </is>
       </c>
-      <c r="O281" t="inlineStr">
+      <c r="O281" s="4" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="P281" t="inlineStr">
+      <c r="P281" s="4" t="inlineStr">
         <is>
           <t>Sandwip Bhavon,college road,Halishahor, ctg.</t>
         </is>
       </c>
-      <c r="Q281" t="inlineStr">
+      <c r="Q281" s="4" t="inlineStr">
         <is>
           <t>01789865054</t>
         </is>
       </c>
-      <c r="S281" t="inlineStr">
+      <c r="S281" s="4" t="inlineStr">
         <is>
           <t>halishahar</t>
         </is>
       </c>
     </row>
     <row r="282">
-      <c r="A282" t="n">
+      <c r="A282" s="4" t="n">
         <v>3856</v>
       </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C282" t="inlineStr">
+      <c r="B282" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C282" s="4" t="inlineStr">
         <is>
           <t>01675271093</t>
         </is>
       </c>
-      <c r="D282" t="inlineStr">
+      <c r="D282" s="4" t="inlineStr">
         <is>
           <t>DJG544GCDV</t>
         </is>
       </c>
-      <c r="G282" s="27" t="n">
+      <c r="G282" s="28" t="n">
         <v>46311.7080324074</v>
       </c>
-      <c r="H282" t="inlineStr">
+      <c r="H282" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I282" t="inlineStr">
+      <c r="I282" s="4" t="inlineStr">
         <is>
           <t>Mosaidul Hossain Nihad</t>
         </is>
       </c>
-      <c r="J282" t="inlineStr">
+      <c r="J282" s="4" t="inlineStr">
         <is>
           <t>মোসাইদুল হোসেন নিহাদ</t>
         </is>
       </c>
-      <c r="K282" t="inlineStr">
+      <c r="K282" s="4" t="inlineStr">
         <is>
           <t>Moazzam Hossain Molla</t>
         </is>
       </c>
-      <c r="L282" t="inlineStr">
+      <c r="L282" s="4" t="inlineStr">
         <is>
           <t>Tania Akter</t>
         </is>
       </c>
-      <c r="M282" t="inlineStr">
+      <c r="M282" s="4" t="inlineStr">
         <is>
           <t>Halishahar Cantonment Public School and College</t>
         </is>
       </c>
-      <c r="N282" t="inlineStr">
+      <c r="N282" s="4" t="inlineStr">
         <is>
           <t>Seven</t>
         </is>
       </c>
-      <c r="O282" t="n">
+      <c r="O282" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="P282" t="inlineStr">
+      <c r="P282" s="4" t="inlineStr">
         <is>
           <t>Lane-2, I-Block, Halishahar, Chattogram</t>
         </is>
       </c>
-      <c r="Q282" t="inlineStr">
+      <c r="Q282" s="4" t="inlineStr">
         <is>
           <t>01675271093</t>
         </is>
       </c>
-      <c r="S282" t="inlineStr">
+      <c r="S282" s="4" t="inlineStr">
         <is>
           <t>halishahar</t>
         </is>
       </c>
     </row>
     <row r="283">
-      <c r="A283" t="n">
+      <c r="A283" s="4" t="n">
         <v>3857</v>
       </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C283" t="inlineStr">
+      <c r="B283" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C283" s="4" t="inlineStr">
         <is>
           <t>01723088207</t>
         </is>
       </c>
-      <c r="D283" t="n">
+      <c r="D283" s="4" t="n">
         <v>567</v>
       </c>
-      <c r="G283" s="27" t="n">
+      <c r="G283" s="28" t="n">
         <v>46312.66</v>
       </c>
-      <c r="H283" t="inlineStr">
+      <c r="H283" s="4" t="inlineStr">
         <is>
           <t>Girl</t>
         </is>
       </c>
-      <c r="I283" t="inlineStr">
+      <c r="I283" s="4" t="inlineStr">
         <is>
           <t>Junaira Farisha Islam</t>
         </is>
       </c>
-      <c r="J283" t="inlineStr">
+      <c r="J283" s="4" t="inlineStr">
         <is>
           <t>জুনাইরা ফারিশা ইসলাম</t>
         </is>
       </c>
-      <c r="K283" t="inlineStr">
+      <c r="K283" s="4" t="inlineStr">
         <is>
           <t>Me.Manirul Islam</t>
         </is>
       </c>
-      <c r="L283" t="inlineStr">
+      <c r="L283" s="4" t="inlineStr">
         <is>
           <t>Farhana Akter</t>
         </is>
       </c>
-      <c r="M283" t="inlineStr">
+      <c r="M283" s="4" t="inlineStr">
         <is>
           <t>HCPSC</t>
         </is>
       </c>
-      <c r="N283" t="inlineStr">
+      <c r="N283" s="4" t="inlineStr">
         <is>
           <t>Six</t>
         </is>
       </c>
-      <c r="O283" t="inlineStr">
+      <c r="O283" s="4" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="P283" t="inlineStr">
+      <c r="P283" s="4" t="inlineStr">
         <is>
           <t>House #34, Lane#8, Road# 1,Block# A.Halishahar, ctg</t>
         </is>
       </c>
-      <c r="Q283" t="inlineStr">
+      <c r="Q283" s="4" t="inlineStr">
         <is>
           <t>01838518567</t>
         </is>
       </c>
-      <c r="S283" t="inlineStr">
+      <c r="S283" s="4" t="inlineStr">
         <is>
           <t>halishahar</t>
         </is>
       </c>
     </row>
     <row r="284">
-      <c r="A284" t="n">
+      <c r="A284" s="4" t="n">
         <v>3858</v>
       </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C284" t="inlineStr">
+      <c r="B284" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C284" s="4" t="inlineStr">
         <is>
           <t>01723088207</t>
         </is>
       </c>
-      <c r="D284" t="n">
+      <c r="D284" s="4" t="n">
         <v>567</v>
       </c>
-      <c r="G284" s="27" t="n">
+      <c r="G284" s="28" t="n">
         <v>46312.66608796296</v>
       </c>
-      <c r="H284" t="inlineStr">
+      <c r="H284" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I284" t="inlineStr">
+      <c r="I284" s="4" t="inlineStr">
         <is>
           <t>Zain Riyasat Islam</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr">
+      <c r="J284" s="4" t="inlineStr">
         <is>
           <t>জাইন রিয়াসাত ইসলাম</t>
         </is>
       </c>
-      <c r="K284" t="inlineStr">
+      <c r="K284" s="4" t="inlineStr">
         <is>
           <t>Md.Manirul Islam</t>
         </is>
       </c>
-      <c r="L284" t="inlineStr">
+      <c r="L284" s="4" t="inlineStr">
         <is>
           <t>Farhana Akter</t>
         </is>
       </c>
-      <c r="M284" t="inlineStr">
+      <c r="M284" s="4" t="inlineStr">
         <is>
           <t>HCPSC</t>
         </is>
       </c>
-      <c r="N284" t="inlineStr">
+      <c r="N284" s="4" t="inlineStr">
         <is>
           <t>Four</t>
         </is>
       </c>
-      <c r="O284" t="n">
+      <c r="O284" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="P284" t="inlineStr">
+      <c r="P284" s="4" t="inlineStr">
         <is>
           <t>House #34, Lane#8, Road# 1,Block# A.Halishahar, ctg</t>
         </is>
       </c>
-      <c r="Q284" t="inlineStr">
+      <c r="Q284" s="4" t="inlineStr">
         <is>
           <t>01838518567</t>
         </is>
       </c>
-      <c r="S284" t="inlineStr">
+      <c r="S284" s="4" t="inlineStr">
         <is>
           <t>halishahar</t>
         </is>
       </c>
     </row>
     <row r="285">
-      <c r="A285" t="n">
+      <c r="A285" s="4" t="n">
         <v>3860</v>
       </c>
-      <c r="B285" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="C285" t="inlineStr">
+      <c r="B285" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C285" s="4" t="inlineStr">
         <is>
           <t>01836831037</t>
         </is>
       </c>
-      <c r="D285" t="inlineStr">
+      <c r="D285" s="4" t="inlineStr">
         <is>
           <t>DJI469U57W</t>
         </is>
       </c>
-      <c r="G285" s="27" t="n">
+      <c r="G285" s="28" t="n">
         <v>46313.18204861111</v>
       </c>
-      <c r="H285" t="inlineStr">
+      <c r="H285" s="4" t="inlineStr">
         <is>
           <t>Girl</t>
         </is>
       </c>
-      <c r="I285" t="inlineStr">
+      <c r="I285" s="4" t="inlineStr">
         <is>
           <t>Olin Atfa</t>
         </is>
       </c>
-      <c r="J285" t="inlineStr">
+      <c r="J285" s="4" t="inlineStr">
         <is>
           <t>অলিন আতফা</t>
         </is>
       </c>
-      <c r="K285" t="inlineStr">
+      <c r="K285" s="4" t="inlineStr">
         <is>
           <t>MD. YEASIN ARAFAT</t>
         </is>
       </c>
-      <c r="L285" t="inlineStr">
+      <c r="L285" s="4" t="inlineStr">
         <is>
           <t>SABRIN KHANAM</t>
         </is>
       </c>
-      <c r="M285" t="inlineStr">
+      <c r="M285" s="4" t="inlineStr">
         <is>
           <t>GUL-E-ZAR BEGUM CITY CORP MUSLIM GIRLS HIGH SCHOOL</t>
         </is>
       </c>
-      <c r="N285" t="inlineStr">
+      <c r="N285" s="4" t="inlineStr">
         <is>
           <t>Seven</t>
         </is>
       </c>
-      <c r="O285" t="n">
+      <c r="O285" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="P285" t="inlineStr">
+      <c r="P285" s="4" t="inlineStr">
         <is>
           <t>DC road , chawkbazar, Chittagong</t>
         </is>
       </c>
-      <c r="Q285" t="inlineStr">
+      <c r="Q285" s="4" t="inlineStr">
         <is>
           <t>01866358979</t>
         </is>
       </c>
-      <c r="S285" t="inlineStr">
+      <c r="S285" s="4" t="inlineStr">
         <is>
           <t>dewanhat</t>
         </is>
       </c>
     </row>
     <row r="286">
-      <c r="A286" t="n">
+      <c r="A286" s="4" t="n">
         <v>3861</v>
       </c>
-      <c r="B286" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="E286" t="inlineStr">
+      <c r="B286" s="4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E286" s="4" t="inlineStr">
         <is>
           <t>01722212464</t>
         </is>
       </c>
-      <c r="F286" t="inlineStr">
+      <c r="F286" s="4" t="inlineStr">
         <is>
           <t>766HHM4N</t>
         </is>
       </c>
-      <c r="G286" s="27" t="n">
+      <c r="G286" s="28" t="n">
         <v>46315.56190972222</v>
       </c>
-      <c r="H286" t="inlineStr">
+      <c r="H286" s="4" t="inlineStr">
         <is>
           <t>Boy</t>
         </is>
       </c>
-      <c r="I286" t="inlineStr">
+      <c r="I286" s="4" t="inlineStr">
         <is>
           <t>AFSAN NAZRUL AR-RAFI</t>
         </is>
       </c>
-      <c r="J286" t="inlineStr">
+      <c r="J286" s="4" t="inlineStr">
         <is>
           <t>আফসান নজরুল আর-রাফি</t>
         </is>
       </c>
-      <c r="K286" t="inlineStr">
+      <c r="K286" s="4" t="inlineStr">
         <is>
           <t>MD. NAZRUL ISLAM</t>
         </is>
       </c>
-      <c r="L286" t="inlineStr">
+      <c r="L286" s="4" t="inlineStr">
         <is>
           <t>KANICH FATIMA</t>
         </is>
       </c>
-      <c r="M286" t="inlineStr">
+      <c r="M286" s="4" t="inlineStr">
         <is>
           <t>Ispahani Public School &amp; College</t>
         </is>
       </c>
-      <c r="N286" t="inlineStr">
+      <c r="N286" s="4" t="inlineStr">
         <is>
           <t>Five</t>
         </is>
       </c>
-      <c r="O286" t="n">
+      <c r="O286" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="P286" t="inlineStr">
+      <c r="P286" s="4" t="inlineStr">
         <is>
           <t>Kusumbag R/A, Goribullah shah majar, Khulshi, Chattogram</t>
         </is>
       </c>
-      <c r="Q286" t="inlineStr">
+      <c r="Q286" s="4" t="inlineStr">
         <is>
           <t>01953031941</t>
         </is>
       </c>
-      <c r="S286" t="inlineStr">
+      <c r="S286" s="4" t="inlineStr">
         <is>
           <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>3695</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>01911246556</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>DIO2U2GM3E</t>
+        </is>
+      </c>
+      <c r="G287" s="28" t="n">
+        <v>46289.56113425926</v>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>ZAFIRA AHMED</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>জাফিরা আহমদ</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>ZABED AHMED</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>ZAKIA FARHANA</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Silver Bells Kindergarten &amp; Girls' High School</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>SIX</t>
+        </is>
+      </c>
+      <c r="O287" t="n">
+        <v>11</v>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>D6, HOUSE NO-03, LANE NO-02, ROAD NO-01, BLOCK-G, HALISHAHAR H/E, HALISHAHAR, CHATTOGRAM</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>01911246556</t>
+        </is>
+      </c>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>3786</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>01815511550</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Humaira Jahan</t>
+        </is>
+      </c>
+      <c r="G288" s="28" t="n">
+        <v>46296.55094907407</v>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Humaira Jahan Rejum</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>হুমায়রা জাহান রিজুম</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>MD Shahjahan</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>Mrs Halima Khatun</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Kattali Ideal Kinder Garten And High School</t>
+        </is>
+      </c>
+      <c r="N288" t="n">
+        <v>9</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>North Kattali, Ina Gazi Bari, Akborshah, Chittagong</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>01815511550</t>
+        </is>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>3834</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>01820293583</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>DJ91NISEWL</t>
+        </is>
+      </c>
+      <c r="G289" s="28" t="n">
+        <v>46305.30952546297</v>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Faria Jamal</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>ফারিয়া জামাল</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>MD Jamal Uddin</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Goal Nahar</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>Feni Govt Girls High School</t>
+        </is>
+      </c>
+      <c r="N289" t="n">
+        <v>9</v>
+      </c>
+      <c r="O289" t="n">
+        <v>16</v>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>Nazir road,Feni</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>01820293583</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>3862</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>01712386612</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>766LJLCV</t>
+        </is>
+      </c>
+      <c r="G290" s="28" t="n">
+        <v>46316.26416666667</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>MD. ATIQUL ALAM RAFI</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>মোঃ আতিকুল আলম রাফি</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>RUMAN</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>MONIRA</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>PRAVATI MADDHYAMIK SHIKKHA NIKETON</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>FIVE</t>
+        </is>
+      </c>
+      <c r="O290" t="n">
+        <v>53</v>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>CHOWDHURY VILLA, BLOCK-B, KAIBALYADHAM R/A, FIROZSHAH, CHATTOGRAM</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>01712386612</t>
+        </is>
+      </c>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>3863</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>01712386612</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>766LNA43</t>
+        </is>
+      </c>
+      <c r="G291" s="28" t="n">
+        <v>46316.27618055556</v>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>TAHASAN KHONDOKAR</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>তাহসান খন্দকার</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>MD IMRAN</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>SUFIYA JAMAN JANY</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>PRAVATI MADDHYAMIK SHIKKHA NIKETON</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>FIVE</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>CDA R/A, UTTAR KATTALI, CHATTOGRAM CITY CORPORATION, CTG.</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>01866605785</t>
+        </is>
+      </c>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>3864</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>01805414488</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>DJL3C1P8XJ</t>
+        </is>
+      </c>
+      <c r="G292" s="28" t="n">
+        <v>46316.37563657408</v>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Afra Anwar</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>আফরা আনোয়ার</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>MD. Anwar Hossain</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Nazreen Akhter</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Dr. Khastagir Govt. Girls High School</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>5,</t>
+        </is>
+      </c>
+      <c r="O292" t="n">
+        <v>11</v>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>Bahaddarhat, chattogram</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>01816611258</t>
+        </is>
+      </c>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>3865</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>01723088207</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>DIK30j1E2N</t>
+        </is>
+      </c>
+      <c r="G293" s="28" t="n">
+        <v>46316.45472222222</v>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Nusaiba Tarnnum</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>নুসাইবা তারান্নুম</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>Ismail jabiullah</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Mobassera Begum</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Nasirabad gov. girls high school.</t>
+        </is>
+      </c>
+      <c r="N293" t="n">
+        <v>8</v>
+      </c>
+      <c r="O293" t="n">
+        <v>41</v>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>Kunjachaya r/a, Bayezid Bostami</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>01755792267</t>
+        </is>
+      </c>
+      <c r="S293" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>3866</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>01817747042</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>DJL9CGDGA7</t>
+        </is>
+      </c>
+      <c r="G294" s="28" t="n">
+        <v>46316.54778935185</v>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Samaira Muntaha Arha</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>সামাইরা মুনতাহা আরহা</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>Shahadat Hossain</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Taohida Akter</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>Halishahar Cantonment public school and college</t>
+        </is>
+      </c>
+      <c r="N294" t="n">
+        <v>6</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>Halishahar Green View R/A road no 3</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>01678060130</t>
+        </is>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>3867</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>01818022749</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>DJL6CIIU8U</t>
+        </is>
+      </c>
+      <c r="G295" s="28" t="n">
+        <v>46316.56142361111</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Mohammed Ahrar Rahman</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>মুহাম্মদ আহরার রহমান</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>Mohammed Khalilur Rahman</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Farida Yasmin</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>Chattogram Collegiate school</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="O295" t="n">
+        <v>51</v>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>Amena Villa.3253/G.Banarupa R/A, Loharpool Saraipara Pahartali Chattogram</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>01818022749</t>
+        </is>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>halishahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>3868</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>01819107308</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>DJL8CJUJXU</t>
+        </is>
+      </c>
+      <c r="G296" s="28" t="n">
+        <v>46316.57699074074</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Abdullah al farhan</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>আবদুল্লাহ আল ফারহান</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>Ershad Hossain</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Maksura jahan</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>Shah wali ullah institute</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>Seven</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>LIBERTY SQUARE, 349/392 KAPASGOLA CHATTOGRAM</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>01836232866</t>
+        </is>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>3869</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>01581416332</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="G297" s="28" t="n">
+        <v>46316.61653935185</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Jannatul Ferdous</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>জান্নাতুল ফেরদৌস</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>মো. সেলিম উদ্দিন</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>জোসনা আক্তার</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>পূর্ব টাইগারপাস সরকারি প্রাথমিক বিদ্যালয়</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>মতি ঝর্ণা, লালখান বাজার, চট্টগ্রাম ।</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>01577707123</t>
+        </is>
+      </c>
+      <c r="S297" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>3871</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>01981666653</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>DJL1CSTHOL</t>
+        </is>
+      </c>
+      <c r="G298" s="28" t="n">
+        <v>46316.67668981481</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Syed nafis fuad</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>সৈয়দ নাফিস ফুয়াদ</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>Syed Nazmul huda</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Dolna khanom</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Halishar cantonment public school and college</t>
+        </is>
+      </c>
+      <c r="N298" t="n">
+        <v>7</v>
+      </c>
+      <c r="O298" t="n">
+        <v>20</v>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>723,London building,Baitul jannat moshjid lane kadamtali Chattogram</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>01981666653</t>
+        </is>
+      </c>
+      <c r="S298" t="inlineStr">
+        <is>
+          <t>dewanhat</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>3872</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>01571475611</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Mahib sw</t>
+        </is>
+      </c>
+      <c r="G299" s="28" t="n">
+        <v>46316.70928240741</v>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Boy</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Imran Al Noor</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>ইমরান আল নুর</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>Mohammed Noor Uddin</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>Jannatul Ferdous</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>BN School and College</t>
+        </is>
+      </c>
+      <c r="N299" t="n">
+        <v>6</v>
+      </c>
+      <c r="O299" t="n">
+        <v>121</v>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>Fajar ali sarang house, South Halishahar</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>01742688898</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>Patenga</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>3873</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>01878351990</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Ishtiaqe Mahmud</t>
+        </is>
+      </c>
+      <c r="G300" s="28" t="n">
+        <v>46316.72174768519</v>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Girl</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Sabiha Kader Jahin</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>সাবিহা কাদের জাহিন</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>আব্দুল কাদের জিলানী</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>ফরিদা আখতার</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>আলহাজ ইয়াকুব আলী স্কুল এন্ড কলেজ</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>ষষ্ঠ শ্রেণি</t>
+        </is>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>১০</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>বারো কোয়াটার পাহাড়তলী চট্টগ্রাম</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>01854312371</t>
+        </is>
+      </c>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>halishahar</t>
         </is>
       </c>
     </row>

</xml_diff>